<commit_message>
Navair refactored with Scraper class
</commit_message>
<xml_diff>
--- a/I3harris/l3harris_jobs.xlsx
+++ b/I3harris/l3harris_jobs.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,114 +449,145 @@
           <t>URL</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Schedule</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Description(raw)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Electrical or Electro-mechanical Engineering Technologist</t>
+          <t>Composite Technician A</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OTTAWA, ONTARIO</t>
+          <t>HUNTSVILLE, AL</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>84547371872</t>
+          <t>84577974544</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://careers.l3harris.com/en/job/ottawa/electrical-or-electro-mechanical-engineering-technologist/4832/84547371872</t>
+          <t>https://careers.l3harris.com/en/job/huntsville/composite-technician-a/4832/84577974544</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>3rd Shift 9/80 work 9 out of every 14 days – totaling 80 hours worked – and have every other Friday off</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+        &lt;div class="job-buttons"&gt;
+	&lt;a class="button job-apply top" data-job-id="84577974544" data-job-organization-id="4832" data-selector-name="job-apply-link" data-page-type="Job" data-page-name="Job Details" data-override-candidate-card="False" data-delay-url="False" data-apply-url="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26962" href="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26962" rel="nofollow" data-apply-mobile="true"&gt;Apply Now&lt;/a&gt;                &lt;button type="button" class="js-save-job-btn" data-job-id="84577974544" data-org-id="4832" data-job-saved="false" style="display: none;"&gt;Save Job&lt;/button&gt;
+        &lt;/div&gt;
+        &lt;div class="ats-description"&gt;
+            &lt;div class="ats-intro"&gt;
+            &lt;/div&gt;
+            &lt;div class="desc"&gt;
+                &lt;p&gt;L3Harris is dedicated to recruiting and developing high-performing talent who are passionate about what they do. Our employees are unified in a shared dedication to our customers’ mission and quest for professional growth. L3Harris provides an inclusive, engaging environment designed to empower employees and promote work-life success. Fundamental to our culture is an unwavering focus on values, dedication to our communities, and commitment to excellence in everything we do.&lt;/p&gt;&lt;p&gt;L3Harris Technologies is the Trusted Disruptor in the defense industry. With customers’ mission-critical needs always in mind, our employees deliver end-to-end technology solutions connecting the space, air, land, sea and cyber domains in the interest of national security.&lt;/p&gt;&lt;p&gt;&lt;/p&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;&lt;strong&gt;Job Title: Composite Technician A&lt;/strong&gt;&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;&lt;strong&gt;Job Code: 26962&lt;/strong&gt;&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;&lt;strong&gt;Job Location:&amp;nbsp; Huntsville, AL (AMF North location)&lt;/strong&gt;&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;&lt;strong&gt;Job Schedule: 3rd Shift 9/80 work 9 out of every 14 days – totaling 80 hours worked – and have every other Friday off&lt;/strong&gt;&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;&lt;/p&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;&lt;strong&gt;Job Description:&lt;/strong&gt;&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;&lt;span style="color: #000000;"&gt;L3Haris is seeking a Composite Manufacturing Technician to work at our state-of-the-art Advanced Manufacturing Facility (AMF) in Huntsville, AL, which will be our inert manufacturing facility for fabrication and assembly of composite rocket motor hardware.&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;&lt;/p&gt;&lt;p style="text-indent: 0.5pt;"&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;&lt;strong&gt;Essential Functions:&amp;nbsp; &lt;/strong&gt;&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;ul style="margin-bottom: 17.0px;"&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Produce parts, components and final assemblies using composite fabrication, compression molding, metal fabrication, modification, checkout, re-work, quality testing, and assembly utilizing detailed work instructions, schematics, diagrams, layouts or manufacturing test development or diagnostic equipment&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Prepare various components for lay-up, filament winding, cure and post cure using cured and uncured rubber materials and adhesives&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Operation of various machinery and shop equipment which may include but not be limited to filament winders, ovens, autoclaves, manual lathes, CNC lathes, CNC milling centers, manual mills, boring mills, presses, furnaces, mixers, grinders, swages, paint booths, fume hoods and automated welding equipment&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Fabrication and assembly of piece parts into completed sub-assembly using assembly tools&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Perform vacuum bagging and related processes for fabrication and curing composite parts&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Complete structural bonding operations using film adhesives, core materials, and adhesives&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Building of complex layups individually and in small groups&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Insulation of mandrels and composite cases&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Filament winding composite structures&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Cast, cure and machining of sand mandrels&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Facilitate and conduct OJT training of technicians as required&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Troubleshoot processes and identify, modify and/or escalate out of control processes and production escapes&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Ability to work additional shifts as needed&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Coordinate with maintenance, supervision and/or engineers in the set-up and calibration of equipment&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Participate in preventative maintenance activities&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Clean machines, equipment, and work area according to Standard Operating Procedures&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong style="color: #000000; font-family: Verdana, Geneva, sans-serif; font-size: 14.0px;"&gt;Qualifications:&lt;/strong&gt;&lt;/p&gt;&lt;ul style="margin-bottom: 11.0px;"&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;High School Diploma or equivalent with 0-3 years prior experience in Manufacturing&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;span style="color: #ffffff;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;#LI-JC4&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;L3Harris Technologies is proud to be an Equal Opportunity Employer. L3Harris is committed to treating all employees and applicants for employment with respect and dignity and maintaining a workplace that is free from unlawful discrimination. All applicants will be considered for employment without regard to race, color, religion, age, national origin, ancestry, ethnicity, gender (including pregnancy, childbirth, breastfeeding or other related medical conditions), gender identity, gender expression, sexual orientation, marital status, veteran status, disability, genetic information, citizenship status, characteristic or membership in any other group protected by federal, state or local laws. L3Harris maintains a drug-free workplace and performs pre-employment substance abuse testing and background checks, where permitted by law.&lt;/p&gt;&lt;p&gt;Please be aware many of our positions require the ability to obtain a security clearance. Security clearances may only be granted to U.S. citizens. In addition, applicants who accept a conditional offer of employment may be subject to government security investigation(s) and must meet eligibility requirements for access to classified information. &lt;/p&gt;&lt;p&gt;By submitting your resume for this position, you understand and agree that L3Harris Technologies may share your resume, as well as any other related personal information or documentation you provide, with its subsidiaries and affiliated companies for the purpose of considering you for other available positions.&lt;/p&gt;&lt;p&gt;L3Harris Technologies is an E-Verify Employer. Please click here for the E-Verify Poster in &lt;a href="https://www.e-verify.gov/sites/default/files/everify/posters/EVerifyParticipationPoster.pdf" class="external-link" target="_blank" rel="nofollow noopener"&gt;English&lt;/a&gt; or &lt;a href="https://www.e-verify.gov/sites/default/files/everify/posters/EVerifyParticipationPoster.pdf" class="external-link" target="_blank" rel="nofollow noopener"&gt;Spanish&lt;/a&gt;. For information regarding your Right To Work, please click here for &lt;a href="https://www.eeoc.gov/sites/default/files/2022-10/22-088_EEOC_KnowYourRights_10_20.pdf" class="external-link" target="_blank" rel="nofollow noopener"&gt;English&lt;/a&gt; or &lt;a href="https://www.eeoc.gov/sites/default/files/2022-10/22-088_EEOC_KnowYourRightsSp_10_20.pdf" class="external-link" target="_blank" rel="nofollow noopener"&gt;Spanish&lt;/a&gt;.&lt;/p&gt;
+            &lt;/div&gt;
+            &lt;div class="qualifications"&gt;
+            &lt;/div&gt;
+        &lt;/div&gt;
+	&lt;a class="button job-apply bottom" data-job-id="84577974544" data-job-organization-id="4832" data-selector-name="job-apply-link" data-page-type="Job" data-page-name="Job Details" data-override-candidate-card="False" data-delay-url="False" data-apply-url="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26962" href="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26962" rel="nofollow" data-apply-mobile="true"&gt;Apply Now&lt;/a&gt;        
+    </t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>&lt;div class="job-buttons"&gt;
+&lt;a class="button job-apply top" data-job-id="84577974544" data-job-organization-id="4832" data-selector-name="job-apply-link" data-page-type="Job" data-page-name="Job Details" data-override-candidate-card="False" data-delay-url="False" data-apply-url="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26962" href="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26962" rel="nofollow" data-apply-mobile="true"&gt;&lt;/a&gt;                &lt;button type="button" class="js-save-job-btn" data-job-id="84577974544" data-org-id="4832" data-job-saved="false" style="display: none;"&gt;Save Job&lt;/button&gt;
+&lt;/div&gt;
+&lt;div class="ats-description"&gt;
+&lt;div class="ats-intro"&gt;
+&lt;/div&gt;
+&lt;div class="desc"&gt;
+&lt;p&gt;L3Harris is dedicated to recruiting and developing high-performing talent who are passionate about what they do. Our employees are unified in a shared dedication to our customers’ mission and quest for professional growth. L3Harris provides an inclusive, engaging environment designed to empower employees and promote work-life success. Fundamental to our culture is an unwavering focus on values, dedication to our communities, and commitment to excellence in everything we do.&lt;/p&gt;&lt;p&gt;L3Harris Technologies is the Trusted Disruptor in the defense industry. With customers’ mission-critical needs always in mind, our employees deliver end-to-end technology solutions connecting the space, air, land, sea and cyber domains in the interest of national security.&lt;/p&gt;&lt;p&gt;&lt;/p&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;&lt;strong&gt;Job Title: Composite Technician A&lt;/strong&gt;&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;&lt;strong&gt;Job Code: 26962&lt;/strong&gt;&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;&lt;strong&gt;Job Location:&amp;nbsp; Huntsville, AL (AMF North location)&lt;/strong&gt;&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;&lt;strong&gt;Job Schedule: 3rd Shift 9/80 work 9 out of every 14 days – totaling 80 hours worked – and have every other Friday off&lt;/strong&gt;&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;&lt;/p&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;&lt;strong&gt;Job Description:&lt;/strong&gt;&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;&lt;span style="color: #000000;"&gt;L3Haris is seeking a Composite Manufacturing Technician to work at our state-of-the-art Advanced Manufacturing Facility (AMF) in Huntsville, AL, which will be our inert manufacturing facility for fabrication and assembly of composite rocket motor hardware.&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;&lt;/p&gt;&lt;p style="text-indent: 0.5pt;"&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;&lt;strong&gt;Essential Functions:&amp;nbsp; &lt;/strong&gt;&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;ul style="margin-bottom: 17.0px;"&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Produce parts, components and final assemblies using composite fabrication, compression molding, metal fabrication, modification, checkout, re-work, quality testing, and assembly utilizing detailed work instructions, schematics, diagrams, layouts or manufacturing test development or diagnostic equipment&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Prepare various components for lay-up, filament winding, cure and post cure using cured and uncured rubber materials and adhesives&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Operation of various machinery and shop equipment which may include but not be limited to filament winders, ovens, autoclaves, manual lathes, CNC lathes, CNC milling centers, manual mills, boring mills, presses, furnaces, mixers, grinders, swages, paint booths, fume hoods and automated welding equipment&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Fabrication and assembly of piece parts into completed sub-assembly using assembly tools&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Perform vacuum bagging and related processes for fabrication and curing composite parts&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Complete structural bonding operations using film adhesives, core materials, and adhesives&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Building of complex layups individually and in small groups&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Insulation of mandrels and composite cases&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Filament winding composite structures&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Cast, cure and machining of sand mandrels&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Facilitate and conduct OJT training of technicians as required&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Troubleshoot processes and identify, modify and/or escalate out of control processes and production escapes&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Ability to work additional shifts as needed&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Coordinate with maintenance, supervision and/or engineers in the set-up and calibration of equipment&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Participate in preventative maintenance activities&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;Clean machines, equipment, and work area according to Standard Operating Procedures&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;strong style="color: #000000; font-family: Verdana, Geneva, sans-serif; font-size: 14.0px;"&gt;Qualifications:&lt;/strong&gt;&lt;/p&gt;&lt;ul style="margin-bottom: 11.0px;"&gt;&lt;li&gt;&lt;p&gt;&lt;span style="color: #000000;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;High School Diploma or equivalent with 0-3 years prior experience in Manufacturing&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;/li&gt;&lt;/ul&gt;&lt;p&gt;&lt;span style="color: #ffffff;"&gt;&lt;span style="font-size: 14.0px;"&gt;&lt;span style="font-family: Verdana, Geneva, sans-serif;"&gt;#LI-JC4&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;L3Harris Technologies is proud to be an Equal Opportunity Employer. L3Harris is committed to treating all employees and applicants for employment with respect and dignity and maintaining a workplace that is free from unlawful discrimination. All applicants will be considered for employment without regard to race, color, religion, age, national origin, ancestry, ethnicity, gender (including pregnancy, childbirth, breastfeeding or other related medical conditions), gender identity, gender expression, sexual orientation, marital status, veteran status, disability, genetic information, citizenship status, characteristic or membership in any other group protected by federal, state or local laws. L3Harris maintains a drug-free workplace and performs pre-employment substance abuse testing and background checks, where permitted by law.&lt;/p&gt;&lt;p&gt;Please be aware many of our positions require the ability to obtain a security clearance. Security clearances may only be granted to U.S. citizens. In addition, applicants who accept a conditional offer of employment may be subject to government security investigation(s) and must meet eligibility requirements for access to classified information. &lt;/p&gt;&lt;p&gt;By submitting your resume for this position, you understand and agree that L3Harris Technologies may share your resume, as well as any other related personal information or documentation you provide, with its subsidiaries and affiliated companies for the purpose of considering you for other available positions.&lt;/p&gt;&lt;p&gt;L3Harris Technologies is an E-Verify Employer. Please click here for the E-Verify Poster in &lt;a href="https://www.e-verify.gov/sites/default/files/everify/posters/EVerifyParticipationPoster.pdf" class="external-link" target="_blank" rel="nofollow noopener"&gt;English&lt;/a&gt; or &lt;a href="https://www.e-verify.gov/sites/default/files/everify/posters/EVerifyParticipationPoster.pdf" class="external-link" target="_blank" rel="nofollow noopener"&gt;Spanish&lt;/a&gt;. For information regarding your Right To Work, please click here for &lt;a href="https://www.eeoc.gov/sites/default/files/2022-10/22-088_EEOC_KnowYourRights_10_20.pdf" class="external-link" target="_blank" rel="nofollow noopener"&gt;English&lt;/a&gt; or &lt;a href="https://www.eeoc.gov/sites/default/files/2022-10/22-088_EEOC_KnowYourRightsSp_10_20.pdf" class="external-link" target="_blank" rel="nofollow noopener"&gt;Spanish&lt;/a&gt;.&lt;/p&gt;
+&lt;/div&gt;
+&lt;div class="qualifications"&gt;
+&lt;/div&gt;
+&lt;/div&gt;
+&lt;a class="button job-apply bottom" data-job-id="84577974544" data-job-organization-id="4832" data-selector-name="job-apply-link" data-page-type="Job" data-page-name="Job Details" data-override-candidate-card="False" data-delay-url="False" data-apply-url="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26962" href="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26962" rel="nofollow" data-apply-mobile="true"&gt;&lt;/a&gt;</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Trade Compliance Sr. Specialist - Licensing</t>
+          <t>Electrical or Electro-mechanical Engineering Technologist</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Multiple Locations</t>
+          <t>OTTAWA, ONTARIO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>84466125424</t>
+          <t>84547371872</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://careers.l3harris.com/en/job/melbourne/trade-compliance-sr-specialist-licensing/4832/84466125424</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Corporate Manufacturing Engineering &amp; Front Loading</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>MELBOURNE, FL</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>84393232480</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>https://careers.l3harris.com/en/job/melbourne/corporate-manufacturing-engineering-and-front-loading/4832/84393232480</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Lead, Manufacturing Engineer</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Multiple Locations</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>84424271696</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>https://careers.l3harris.com/en/job/camden/lead-manufacturing-engineer/4832/84424271696</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Sr. Specialist, Trade Compliance (Empowered Official)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>SALT LAKE CITY, UT</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>84466125344</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>https://careers.l3harris.com/en/job/salt-lake-city/sr-specialist-trade-compliance-empowered-official/4832/84466125344</t>
+          <t>https://careers.l3harris.com/en/job/ottawa/electrical-or-electro-mechanical-engineering-technologist/4832/84547371872</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+        &lt;div class="job-buttons"&gt;
+	&lt;a class="button job-apply top" data-job-id="84547371872" data-job-organization-id="4832" data-selector-name="job-apply-link" data-page-type="Job" data-page-name="Job Details" data-override-candidate-card="False" data-delay-url="False" data-apply-url="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26992" href="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26992" rel="nofollow" data-apply-mobile="true" data-url-type="0" style="pointer-events: auto;"&gt;Apply Now&lt;/a&gt;                &lt;button type="button" class="js-save-job-btn" data-job-id="84547371872" data-org-id="4832" data-job-saved="false" style="display: none;"&gt;Save Job&lt;/button&gt;
+        &lt;/div&gt;
+        &lt;div class="ats-description"&gt;
+            &lt;div class="ats-intro"&gt;
+            &lt;/div&gt;
+            &lt;div class="desc"&gt;
+                &lt;p&gt;L3Harris is dedicated to recruiting and developing high-performing talent who are passionate about what they do. Our employees are unified in a shared dedication to our customers’ mission and quest for professional growth. L3Harris provides an inclusive, engaging environment designed to empower employees and promote work-life success. Fundamental to our culture is an unwavering focus on values, dedication to our communities, and commitment to excellence in everything we do.&lt;/p&gt;&lt;p&gt;L3Harris Technologies is the Trusted Disruptor in the defense industry. With customers’ mission-critical needs always in mind, our employees deliver end-to-end technology solutions connecting the space, air, land, sea and cyber domains in the interest of national security.&lt;/p&gt;&lt;p&gt;&lt;/p&gt;&lt;p class="CxSpFirst"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;&lt;b&gt;About your next Challenge as an Electrical or Electro-mechanical Engineering Technologist&amp;nbsp;&lt;/b&gt;&lt;span class="Style1"&gt;&lt;b&gt;:&lt;/b&gt;&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p class="CxSpMiddle"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;L3Harris Ottawa is seeking a Technician B to join our team. The Technician B will provide support to the production line with unit rework, troubleshooting and assembly.&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p class="CxSpMiddle"&gt;&lt;/p&gt;&lt;p class="CxSpMiddle"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;&lt;b&gt;What will you do: &lt;/b&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Read and interpret documents such as work instructions, safety rules, operating and maintenance instructions&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Assemble mechanical, optical or electrical components and subassemblies following specified work instructions and procedures to ensure finished&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;product meets established operational and cosmetic requirements&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Continuously perform visual inspections of materials for defects and conducts any range of functional tests and cleaning at prescribed intervals to ensure proper operation of various components during assembly&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Report deviations from standard to appropriate resource for review, instruction and authorization and conducts quality inspection at specified intervals&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Perform accurate data and record keeping&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Maintain work area and equipment in a clean and orderly condition and follows prescribed safety procedures&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Cultivate a culture that assures effective cross functional team work&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Perform job duties in a manner that complies with environmental, health and safety regulations, policies and procedures&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Demonstrate ethical and professional behavior in accordance with company values&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;/ul&gt;&lt;p class="CxSpMiddle"&gt;&lt;/p&gt;&lt;p class="CxSpMiddle"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;&lt;b&gt;Required Skills and Experiences:&lt;/b&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;College Diploma or equivalent and a minimum of 4 years of prior relevant experience.&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;/ul&gt;&lt;p style="text-align:justify"&gt;&lt;/p&gt;&lt;p style="text-align:justify"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;&lt;b&gt;Eligibility Criteria (Mandatory):&lt;/b&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;ul&gt;&lt;li style="text-align:justify"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Must be eligible for registration with the&amp;nbsp;&lt;b&gt;Controlled Goods Program&lt;/b&gt;;&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li style="text-align:justify"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Must be eligible to obtain and maintain a government of Canada &lt;b&gt;Reliability&lt;/b&gt; status and &lt;b&gt;Secret Level 2 / NATO Secret&lt;/b&gt;&amp;nbsp;security clearance.&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li style="text-align:justify"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Must be eligible to meet the requirements for &lt;b&gt;U.S. International Traffic in Arms Regulations (ITAR)&lt;/b&gt;.&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;/ul&gt;&lt;p class="CxSpFirst"&gt;&lt;/p&gt;&lt;p class="CxSpLast"&gt;&lt;/p&gt;&lt;p style="text-align:justify"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;L3Harris is proud to be an equal opportunity employer and is committed to treating all of its employees and job applicants with respect and dignity and to maintaining a workplace free from discrimination. Anyone applying for a position will be considered without regard to the following: race, national or ethnic origin, colour, religion, age, nationality, ancestry, ethnicity, gender, sex, sexual orientation, gender identity or expression, marital status, family status, genetic characteristics, disability, citizenship status, or conviction for an offence for which a pardon has been granted or in respect of which a record suspension has been ordered, or any other characteristic that is protected by applicable human rights legislation. &lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p style="text-align:justify"&gt;&lt;/p&gt;&lt;p style="text-align:justify"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;L3Harris maintains a drug-free workplace and conducts pre-employment drug and alcohol testing and background checks, in accordance with applicable law. Such results are only accessible and viewed by individuals at L3Harris who have direct responsibility in the hiring process. If you fail to report for a drug and alcohol test, refuse to undergo such test or test positive for the presence of drugs or alcohol, the hiring process may be concluded or your offer of employment may be rescinded, in L3Harris’ sole discretion.&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;At L3Harris, we foster an inclusive and equitable workplace. L3Harris is committed to treating all employees and applicants for employment with respect and dignity and maintaining a workplace that is free from unlawful discrimination. For applicants with disabilities, we will provide you with accommodation so that you have what you need in order to be at your best.&lt;/p&gt;&lt;p&gt;L3Harris performs background checks prior to employment as all applicants must be eligible for registration with the Controlled Goods Program and obtain and maintain a positive security assessment. Some positions may require a government of Canada “Reliability” status and/or Level 2 (Secret) security clearance. In addition, L3Harris performs pre-employment substance abuse testing where required.&lt;/p&gt;
+            &lt;/div&gt;
+            &lt;div class="qualifications"&gt;
+            &lt;/div&gt;
+        &lt;/div&gt;
+	&lt;a class="button job-apply bottom" data-job-id="84547371872" data-job-organization-id="4832" data-selector-name="job-apply-link" data-page-type="Job" data-page-name="Job Details" data-override-candidate-card="False" data-delay-url="False" data-apply-url="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26992" href="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26992" rel="nofollow" data-apply-mobile="true" data-url-type="0" style="pointer-events: auto;"&gt;Apply Now&lt;/a&gt;        
+    </t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>&lt;div class="job-buttons"&gt;
+&lt;a class="button job-apply top" data-job-id="84547371872" data-job-organization-id="4832" data-selector-name="job-apply-link" data-page-type="Job" data-page-name="Job Details" data-override-candidate-card="False" data-delay-url="False" data-apply-url="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26992" href="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26992" rel="nofollow" data-apply-mobile="true" data-url-type="0" style="pointer-events: auto;"&gt;&lt;/a&gt;                &lt;button type="button" class="js-save-job-btn" data-job-id="84547371872" data-org-id="4832" data-job-saved="false" style="display: none;"&gt;Save Job&lt;/button&gt;
+&lt;/div&gt;
+&lt;div class="ats-description"&gt;
+&lt;div class="ats-intro"&gt;
+&lt;/div&gt;
+&lt;div class="desc"&gt;
+&lt;p&gt;L3Harris is dedicated to recruiting and developing high-performing talent who are passionate about what they do. Our employees are unified in a shared dedication to our customers’ mission and quest for professional growth. L3Harris provides an inclusive, engaging environment designed to empower employees and promote work-life success. Fundamental to our culture is an unwavering focus on values, dedication to our communities, and commitment to excellence in everything we do.&lt;/p&gt;&lt;p&gt;L3Harris Technologies is the Trusted Disruptor in the defense industry. With customers’ mission-critical needs always in mind, our employees deliver end-to-end technology solutions connecting the space, air, land, sea and cyber domains in the interest of national security.&lt;/p&gt;&lt;p&gt;&lt;/p&gt;&lt;p class="CxSpFirst"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;&lt;b&gt;About your next Challenge as an Electrical or Electro-mechanical Engineering Technologist&amp;nbsp;&lt;/b&gt;&lt;span class="Style1"&gt;&lt;b&gt;:&lt;/b&gt;&lt;/span&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p class="CxSpMiddle"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;L3Harris Ottawa is seeking a Technician B to join our team. The Technician B will provide support to the production line with unit rework, troubleshooting and assembly.&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p class="CxSpMiddle"&gt;&lt;/p&gt;&lt;p class="CxSpMiddle"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;&lt;b&gt;What will you do: &lt;/b&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Read and interpret documents such as work instructions, safety rules, operating and maintenance instructions&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Assemble mechanical, optical or electrical components and subassemblies following specified work instructions and procedures to ensure finished&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;product meets established operational and cosmetic requirements&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Continuously perform visual inspections of materials for defects and conducts any range of functional tests and cleaning at prescribed intervals to ensure proper operation of various components during assembly&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Report deviations from standard to appropriate resource for review, instruction and authorization and conducts quality inspection at specified intervals&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Perform accurate data and record keeping&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Maintain work area and equipment in a clean and orderly condition and follows prescribed safety procedures&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Cultivate a culture that assures effective cross functional team work&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Perform job duties in a manner that complies with environmental, health and safety regulations, policies and procedures&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Demonstrate ethical and professional behavior in accordance with company values&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;/ul&gt;&lt;p class="CxSpMiddle"&gt;&lt;/p&gt;&lt;p class="CxSpMiddle"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;&lt;b&gt;Required Skills and Experiences:&lt;/b&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;College Diploma or equivalent and a minimum of 4 years of prior relevant experience.&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;/ul&gt;&lt;p style="text-align:justify"&gt;&lt;/p&gt;&lt;p style="text-align:justify"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;&lt;b&gt;Eligibility Criteria (Mandatory):&lt;/b&gt;&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;ul&gt;&lt;li style="text-align:justify"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Must be eligible for registration with the&amp;nbsp;&lt;b&gt;Controlled Goods Program&lt;/b&gt;;&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li style="text-align:justify"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Must be eligible to obtain and maintain a government of Canada &lt;b&gt;Reliability&lt;/b&gt; status and &lt;b&gt;Secret Level 2 / NATO Secret&lt;/b&gt;&amp;nbsp;security clearance.&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;li style="text-align:justify"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;Must be eligible to meet the requirements for &lt;b&gt;U.S. International Traffic in Arms Regulations (ITAR)&lt;/b&gt;.&lt;/span&gt;&lt;/span&gt;&lt;/li&gt;&lt;/ul&gt;&lt;p class="CxSpFirst"&gt;&lt;/p&gt;&lt;p class="CxSpLast"&gt;&lt;/p&gt;&lt;p style="text-align:justify"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;L3Harris is proud to be an equal opportunity employer and is committed to treating all of its employees and job applicants with respect and dignity and to maintaining a workplace free from discrimination. Anyone applying for a position will be considered without regard to the following: race, national or ethnic origin, colour, religion, age, nationality, ancestry, ethnicity, gender, sex, sexual orientation, gender identity or expression, marital status, family status, genetic characteristics, disability, citizenship status, or conviction for an offence for which a pardon has been granted or in respect of which a record suspension has been ordered, or any other characteristic that is protected by applicable human rights legislation. &lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p style="text-align:justify"&gt;&lt;/p&gt;&lt;p style="text-align:justify"&gt;&lt;span style="font-size:14.0px"&gt;&lt;span style="font-family:Verdana,Geneva,sans-serif"&gt;L3Harris maintains a drug-free workplace and conducts pre-employment drug and alcohol testing and background checks, in accordance with applicable law. Such results are only accessible and viewed by individuals at L3Harris who have direct responsibility in the hiring process. If you fail to report for a drug and alcohol test, refuse to undergo such test or test positive for the presence of drugs or alcohol, the hiring process may be concluded or your offer of employment may be rescinded, in L3Harris’ sole discretion.&lt;/span&gt;&lt;/span&gt;&lt;/p&gt;&lt;p&gt;At L3Harris, we foster an inclusive and equitable workplace. L3Harris is committed to treating all employees and applicants for employment with respect and dignity and maintaining a workplace that is free from unlawful discrimination. For applicants with disabilities, we will provide you with accommodation so that you have what you need in order to be at your best.&lt;/p&gt;&lt;p&gt;L3Harris performs background checks prior to employment as all applicants must be eligible for registration with the Controlled Goods Program and obtain and maintain a positive security assessment. Some positions may require a government of Canada “Reliability” status and/or Level 2 (Secret) security clearance. In addition, L3Harris performs pre-employment substance abuse testing where required.&lt;/p&gt;
+&lt;/div&gt;
+&lt;div class="qualifications"&gt;
+&lt;/div&gt;
+&lt;/div&gt;
+&lt;a class="button job-apply bottom" data-job-id="84547371872" data-job-organization-id="4832" data-selector-name="job-apply-link" data-page-type="Job" data-page-name="Job Details" data-override-candidate-card="False" data-delay-url="False" data-apply-url="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26992" href="https://career-hcm20.ns2cloud.com/careers?company=L3HHCM20&amp;amp;clientId=jobs2web&amp;amp;career_ns=job_application&amp;amp;career_job_req_id=26992" rel="nofollow" data-apply-mobile="true" data-url-type="0" style="pointer-events: auto;"&gt;&lt;/a&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>